<commit_message>
build: rebuild all 13 workbooks from the complete course and pin byte-identical rebuilds
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EaSHWrLVjcRFSEFZAsuapw
</commit_message>
<xml_diff>
--- a/workbooks/01 Shortcuts 1 - Navigate and Select.xlsx
+++ b/workbooks/01 Shortcuts 1 - Navigate and Select.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="487">
   <si>
     <t>Challenge</t>
   </si>
@@ -1718,12 +1718,6 @@
   </si>
   <si>
     <t>F7</t>
-  </si>
-  <si>
-    <t>Boss F8</t>
-  </si>
-  <si>
-    <t>F8</t>
   </si>
   <si>
     <t>BOSS MISSIONS</t>
@@ -2720,7 +2714,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2730,12 +2724,12 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -2745,32 +2739,32 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="5" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="5" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="5" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="5" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="5" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="4" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -2780,30 +2774,30 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>429</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>430</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>431</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="7" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C13" s="9" cm="1" t="str">
         <f t="array" ref="C13">SUM('S1-1 Warp Zones'!$G$17:$G$33)&amp;" / 130"</f>
@@ -2818,15 +2812,15 @@
         <v>NEW</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="7" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="C14" s="9" cm="1" t="str">
         <f t="array" ref="C14">SUM('S1-2 Teleport'!$G$15:$G$39)&amp;" / 180"</f>
@@ -2841,15 +2835,15 @@
         <v>NEW</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="7" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="C15" s="9" cm="1" t="str">
         <f t="array" ref="C15">SUM('S1-3 Lasso'!$G$14:$G$37)&amp;" / 170"</f>
@@ -2864,15 +2858,15 @@
         <v>NEW</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="7" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C16" s="9" cm="1" t="str">
         <f t="array" ref="C16">SUM('S1-4 Grab'!$G$13:$G$32)&amp;" / 130"</f>
@@ -2887,56 +2881,56 @@
         <v>NEW</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>443</v>
+      </c>
+      <c r="C17" s="9" cm="1" t="str">
+        <f t="array" ref="C17">SUM(Boss!$G$14:$G$34)&amp;" / 170"</f>
+        <v>0 / 170</v>
+      </c>
+      <c r="D17" s="10" cm="1" t="str">
+        <f t="array" ref="D17">IF(SUM(Boss!$G$14:$G$34)&gt;=170,"★★★",IF(SUM(Boss!$G$14:$G$34)&gt;=170*0.8,"★★☆",IF(SUM(Boss!$G$14:$G$34)&gt;=170*0.5,"★☆☆","☆☆☆")))</f>
+        <v>☆☆☆</v>
+      </c>
+      <c r="E17" s="9" cm="1" t="str">
+        <f t="array" ref="E17">IF(Boss!$C$10="OPEN",IF(SUM(Boss!$G$14:$G$34)&gt;=170*0.5,"DEFEATED","OPEN"),"LOCKED")</f>
+        <v>LOCKED</v>
+      </c>
+      <c r="F17" s="11" t="s">
         <v>444</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>445</v>
-      </c>
-      <c r="C17" s="9" cm="1" t="str">
-        <f t="array" ref="C17">SUM(Boss!$G$14:$G$35)&amp;" / 180"</f>
-        <v>0 / 180</v>
-      </c>
-      <c r="D17" s="10" cm="1" t="str">
-        <f t="array" ref="D17">IF(SUM(Boss!$G$14:$G$35)&gt;=180,"★★★",IF(SUM(Boss!$G$14:$G$35)&gt;=180*0.8,"★★☆",IF(SUM(Boss!$G$14:$G$35)&gt;=180*0.5,"★☆☆","☆☆☆")))</f>
-        <v>☆☆☆</v>
-      </c>
-      <c r="E17" s="9" cm="1" t="str">
-        <f t="array" ref="E17">IF(Boss!$C$10="OPEN",IF(SUM(Boss!$G$14:$G$35)&gt;=180*0.5,"DEFEATED","OPEN"),"LOCKED")</f>
-        <v>LOCKED</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="7" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B19" s="12" cm="1" t="str">
-        <f t="array" ref="B19">(SUM('S1-1 Warp Zones'!$G$17:$G$33)+SUM('S1-2 Teleport'!$G$15:$G$39)+SUM('S1-3 Lasso'!$G$14:$G$37)+SUM('S1-4 Grab'!$G$13:$G$32)+SUM(Boss!$G$14:$G$35))&amp;" / 790"</f>
-        <v>0 / 790</v>
+        <f t="array" ref="B19">(SUM('S1-1 Warp Zones'!$G$17:$G$33)+SUM('S1-2 Teleport'!$G$15:$G$39)+SUM('S1-3 Lasso'!$G$14:$G$37)+SUM('S1-4 Grab'!$G$13:$G$32)+SUM(Boss!$G$14:$G$34))&amp;" / 780"</f>
+        <v>0 / 780</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="7" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B20" s="12" cm="1" t="str">
-        <f t="array" ref="B20">_xlfn.LET(_xlpm.p,(SUM('S1-1 Warp Zones'!$G$17:$G$33)+SUM('S1-2 Teleport'!$G$15:$G$39)+SUM('S1-3 Lasso'!$G$14:$G$37)+SUM('S1-4 Grab'!$G$13:$G$32)+SUM(Boss!$G$14:$G$35))/790,IF(AND(_xlpm.p&gt;=1,ISNUMBER(Boss!$C$8),Boss!$C$8&lt;=10),"S",IF(_xlpm.p&gt;=0.9,"A",IF(_xlpm.p&gt;=0.75,"B",IF(_xlpm.p&gt;=0.5,"C","D")))))</f>
+        <f t="array" ref="B20">_xlfn.LET(_xlpm.p,(SUM('S1-1 Warp Zones'!$G$17:$G$33)+SUM('S1-2 Teleport'!$G$15:$G$39)+SUM('S1-3 Lasso'!$G$14:$G$37)+SUM('S1-4 Grab'!$G$13:$G$32)+SUM(Boss!$G$14:$G$34))/780,IF(AND(_xlpm.p&gt;=1,ISNUMBER(Boss!$C$8),Boss!$C$8&lt;=10),"S",IF(_xlpm.p&gt;=0.9,"A",IF(_xlpm.p&gt;=0.75,"B",IF(_xlpm.p&gt;=0.5,"C","D")))))</f>
         <v>D</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="7" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B21" s="12" cm="1" t="str">
         <f t="array" ref="B21">IF(ISNUMBER(Boss!$C$8),Boss!$C$8&amp;" min (par 10)","—")</f>
@@ -2945,7 +2939,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="7" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B22" s="12" cm="1" t="str">
         <f t="array" ref="B22">IFERROR(INDEX($A$13:$A$16,MATCH("☆☆☆",$D$13:$D$16,0))&amp;" "&amp;INDEX($B$13:$B$16,MATCH("☆☆☆",$D$13:$D$16,0)),IF(Boss!$C$10="OPEN","the Boss","All clear! Aim for rank S"))</f>
@@ -2954,7 +2948,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="13" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -2977,7 +2971,7 @@
     <tabColor rgb="FFB8860B"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -2991,7 +2985,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3002,20 +2996,20 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="26" customHeight="1">
       <c r="A3" s="14" cm="1" t="str">
-        <f t="array" ref="A3">"SCORE "&amp;TEXT(SUM($G$14:$G$35),"0000")&amp;" / 0180"</f>
-        <v>SCORE 0000 / 0180</v>
+        <f t="array" ref="A3">"SCORE "&amp;TEXT(SUM($G$14:$G$34),"0000")&amp;" / 0170"</f>
+        <v>SCORE 0000 / 0170</v>
       </c>
       <c r="C3" s="15" cm="1" t="str">
-        <f t="array" ref="C3">IF(SUM($G$14:$G$35)&gt;=180,"★★★",IF(SUM($G$14:$G$35)&gt;=180*0.8,"★★☆",IF(SUM($G$14:$G$35)&gt;=180*0.5,"★☆☆","☆☆☆")))</f>
+        <f t="array" ref="C3">IF(SUM($G$14:$G$34)&gt;=170,"★★★",IF(SUM($G$14:$G$34)&gt;=170*0.8,"★★☆",IF(SUM($G$14:$G$34)&gt;=170*0.5,"★☆☆","☆☆☆")))</f>
         <v>☆☆☆</v>
       </c>
       <c r="D3" s="16" cm="1" t="str">
-        <f t="array" ref="D3">REPT("█",ROUND(10*SUM($G$14:$G$35)/180,0))&amp;REPT("░",10-ROUND(10*SUM($G$14:$G$35)/180,0))&amp;"  "&amp;TEXT(SUM($G$14:$G$35)/180,"0%")</f>
+        <f t="array" ref="D3">REPT("█",ROUND(10*SUM($G$14:$G$34)/170,0))&amp;REPT("░",10-ROUND(10*SUM($G$14:$G$34)/170,0))&amp;"  "&amp;TEXT(SUM($G$14:$G$34)/170,"0%")</f>
         <v>░░░░░░░░░░  0%</v>
       </c>
     </row>
@@ -3267,74 +3261,74 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="35.5" customHeight="1">
-      <c r="A21" s="18" t="s">
+    <row r="22" spans="1:7" ht="22" customHeight="1">
+      <c r="A22" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="B23" s="11" t="s">
         <v>384</v>
       </c>
-      <c r="B21" s="31" cm="1" t="str">
-        <f t="array" ref="B21">IF($C$10="OPEN","Which key opens the Go To box?  (from S1-2 Teleport)","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="35.5" customHeight="1">
+      <c r="A25" s="18" t="s">
+        <v>387</v>
+      </c>
+      <c r="B25" s="31" cm="1" t="str">
+        <f t="array" ref="B25">IF($C$10="OPEN","In the Boss Arena, click B6 and press Ctrl+↓. Type the word at the end of the long trail.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
-      <c r="C21" s="21"/>
-      <c r="D21" s="22" cm="1" t="str">
-        <f t="array" ref="D21">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$21,IF(TRIM(_xlpm.a&amp;"")="","",IF(OR(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(UPPER(_xlpm.a)," ",""),"CONTROL","CTRL"),"CTL","CTRL"),"ESCAPE","ESC"),"RETURN","ENTER"),"PAGEDOWN","PGDN"),"PGDOWN","PGDN"),"PAGEUP","PGUP"),"ARROWKEYS","ARROW"),"ARROWKEY","ARROW"),"ARROWS","ARROW"),"DOWNARROW","DOWN"),"UPARROW","UP"),"LEFTARROW","LEFT"),"RIGHTARROW","RIGHT"),"ARROWDOWN","DOWN"),"ARROWUP","UP"),"ARROWLEFT","LEFT"),"ARROWRIGHT","RIGHT"),"↓","DOWN"),"↑","UP"),"←","LEFT"),"→","RIGHT"),"SPACEBAR","SPACE"),"−","-"),"MINUS","-"),"PLUS","+")=Key!$E$70:$F$70),"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
+      <c r="C25" s="21"/>
+      <c r="D25" s="22" cm="1" t="str">
+        <f t="array" ref="D25">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$25,IF(TRIM(_xlpm.a&amp;"")="","",IF(SUBSTITUTE(SUBSTITUTE(UPPER(_xlpm.a&amp;"")," ",""),"$","")=Key!$C$70,"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
         <v>LOCKED</v>
       </c>
-      <c r="E21" s="23"/>
-      <c r="F21" s="24" cm="1" t="str">
-        <f t="array" ref="F21">IF(E21="Show hint",Key!$B$70,"")</f>
+      <c r="E25" s="23"/>
+      <c r="F25" s="24" cm="1" t="str">
+        <f t="array" ref="F25">IF(E25="Show hint",Key!$B$70,"")</f>
         <v/>
       </c>
-      <c r="G21" s="25" cm="1">
-        <f t="array" ref="G21">IF(LEFT(D21,1)="✔",IF(E21="Show hint",5,10),0)</f>
+      <c r="G25" s="25" cm="1">
+        <f t="array" ref="G25">IF(LEFT(D25,1)="✔",IF(E25="Show hint",5,10),0)</f>
         <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="22" customHeight="1">
-      <c r="A23" s="4" t="s">
-        <v>385</v>
-      </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="B24" s="11" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="35.5" customHeight="1">
       <c r="A26" s="18" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B26" s="31" cm="1" t="str">
-        <f t="array" ref="B26">IF($C$10="OPEN","In the Boss Arena, click B6 and press Ctrl+↓. Type the word at the end of the long trail.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B26">IF($C$10="OPEN","Click D6 and keep pressing Ctrl+↓ across the gaps. Type the word you reach.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C26" s="21"/>
@@ -3354,10 +3348,10 @@
     </row>
     <row r="27" spans="1:7" ht="35.5" customHeight="1">
       <c r="A27" s="18" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B27" s="31" cm="1" t="str">
-        <f t="array" ref="B27">IF($C$10="OPEN","Click D6 and keep pressing Ctrl+↓ across the gaps. Type the word you reach.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B27">IF($C$10="OPEN","Press F5, go to J1200, then press Ctrl+→. Type the word you land on.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C27" s="21"/>
@@ -3377,10 +3371,10 @@
     </row>
     <row r="28" spans="1:7" ht="35.5" customHeight="1">
       <c r="A28" s="18" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B28" s="31" cm="1" t="str">
-        <f t="array" ref="B28">IF($C$10="OPEN","Press F5, go to J1200, then press Ctrl+→. Type the word you land on.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B28">IF($C$10="OPEN","Press Ctrl+End. Type the word in the last used cell.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C28" s="21"/>
@@ -3400,10 +3394,10 @@
     </row>
     <row r="29" spans="1:7" ht="35.5" customHeight="1">
       <c r="A29" s="18" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B29" s="31" cm="1" t="str">
-        <f t="array" ref="B29">IF($C$10="OPEN","Press Ctrl+End. Type the word in the last used cell.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B29">IF($C$10="OPEN","Press F5 (or Ctrl+G) and go to Q900. Type the word there.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C29" s="21"/>
@@ -3423,15 +3417,15 @@
     </row>
     <row r="30" spans="1:7" ht="35.5" customHeight="1">
       <c r="A30" s="18" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B30" s="31" cm="1" t="str">
-        <f t="array" ref="B30">IF($C$10="OPEN","Press F5 (or Ctrl+G) and go to Q900. Type the word there.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B30">IF($C$10="OPEN","Click F6 and press Ctrl+Shift+↓ to select all ENERGY values. Type the status-bar Sum.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C30" s="21"/>
       <c r="D30" s="22" cm="1" t="str">
-        <f t="array" ref="D30">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$30,IF(TRIM(_xlpm.a&amp;"")="","",IF(SUBSTITUTE(SUBSTITUTE(UPPER(_xlpm.a&amp;"")," ",""),"$","")=Key!$C$75,"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
+        <f t="array" ref="D30">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$30,IF(TRIM(_xlpm.a&amp;"")="","",IF(ABS(IF(ISNUMBER(_xlpm.a),_xlpm.a,VALUE(_xlpm.a&amp;""))-Key!$C$75)&lt;=1E-9*MAX(1,ABS(Key!$C$75)),"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
         <v>LOCKED</v>
       </c>
       <c r="E30" s="23"/>
@@ -3449,7 +3443,7 @@
         <v>404</v>
       </c>
       <c r="B31" s="31" cm="1" t="str">
-        <f t="array" ref="B31">IF($C$10="OPEN","Click F6 and press Ctrl+Shift+↓ to select all ENERGY values. Type the status-bar Sum.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B31">IF($C$10="OPEN","Click any cell in column H and press Ctrl+Space. Type the status-bar Sum.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C31" s="21"/>
@@ -3467,12 +3461,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="35.5" customHeight="1">
+    <row r="32" spans="1:7" ht="51.25" customHeight="1">
       <c r="A32" s="18" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B32" s="31" cm="1" t="str">
-        <f t="array" ref="B32">IF($C$10="OPEN","Click any cell in column H and press Ctrl+Space. Type the status-bar Sum.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B32">IF($C$10="OPEN","Click inside the MOONS table (it starts at L40) and press Ctrl+A once. Type the status-bar Count.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C32" s="21"/>
@@ -3490,17 +3484,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="51.25" customHeight="1">
+    <row r="33" spans="1:7" ht="35.5" customHeight="1">
       <c r="A33" s="18" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B33" s="31" cm="1" t="str">
-        <f t="array" ref="B33">IF($C$10="OPEN","Click inside the MOONS table (it starts at L40) and press Ctrl+A once. Type the status-bar Count.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B33">IF($C$10="OPEN","Click S40 (START) and press Home. Type the word in the cell you land on.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C33" s="21"/>
       <c r="D33" s="22" cm="1" t="str">
-        <f t="array" ref="D33">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$33,IF(TRIM(_xlpm.a&amp;"")="","",IF(ABS(IF(ISNUMBER(_xlpm.a),_xlpm.a,VALUE(_xlpm.a&amp;""))-Key!$C$78)&lt;=1E-9*MAX(1,ABS(Key!$C$78)),"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
+        <f t="array" ref="D33">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$33,IF(TRIM(_xlpm.a&amp;"")="","",IF(SUBSTITUTE(SUBSTITUTE(UPPER(_xlpm.a&amp;"")," ",""),"$","")=Key!$C$78,"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
         <v>LOCKED</v>
       </c>
       <c r="E33" s="23"/>
@@ -3518,12 +3512,12 @@
         <v>412</v>
       </c>
       <c r="B34" s="31" cm="1" t="str">
-        <f t="array" ref="B34">IF($C$10="OPEN","Click S40 (START) and press Home. Type the word in the cell you land on.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
+        <f t="array" ref="B34">IF($C$10="OPEN","Click any cell in row 20 and press Shift+Space. Type the status-bar Count.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
         <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
       </c>
       <c r="C34" s="21"/>
       <c r="D34" s="22" cm="1" t="str">
-        <f t="array" ref="D34">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$34,IF(TRIM(_xlpm.a&amp;"")="","",IF(SUBSTITUTE(SUBSTITUTE(UPPER(_xlpm.a&amp;"")," ",""),"$","")=Key!$C$79,"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
+        <f t="array" ref="D34">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$34,IF(TRIM(_xlpm.a&amp;"")="","",IF(ABS(IF(ISNUMBER(_xlpm.a),_xlpm.a,VALUE(_xlpm.a&amp;""))-Key!$C$79)&lt;=1E-9*MAX(1,ABS(Key!$C$79)),"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
         <v>LOCKED</v>
       </c>
       <c r="E34" s="23"/>
@@ -3536,32 +3530,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="35.5" customHeight="1">
-      <c r="A35" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="B35" s="31" cm="1" t="str">
-        <f t="array" ref="B35">IF($C$10="OPEN","Click any cell in row 20 and press Shift+Space. Type the status-bar Count.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
-        <v>LOCKED · earn ★ on every stage to open the Boss gate</v>
-      </c>
-      <c r="C35" s="21"/>
-      <c r="D35" s="22" cm="1" t="str">
-        <f t="array" ref="D35">IF($C$10="OPEN",IFERROR(_xlfn.LET(_xlpm.a,Boss!$C$35,IF(TRIM(_xlpm.a&amp;"")="","",IF(ABS(IF(ISNUMBER(_xlpm.a),_xlpm.a,VALUE(_xlpm.a&amp;""))-Key!$C$80)&lt;=1E-9*MAX(1,ABS(Key!$C$80)),"✔ CLEAR","✘ TRY AGAIN"))),"✘ TRY AGAIN"),"LOCKED")</f>
-        <v>LOCKED</v>
-      </c>
-      <c r="E35" s="23"/>
-      <c r="F35" s="24" cm="1" t="str">
-        <f t="array" ref="F35">IF(E35="Show hint",Key!$B$80,"")</f>
-        <v/>
-      </c>
-      <c r="G35" s="25" cm="1">
-        <f t="array" ref="G35">IF(LEFT(D35,1)="✔",IF(E35="Show hint",5,10),0)</f>
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0"/>
-  <conditionalFormatting sqref="D14:D35">
+  <conditionalFormatting sqref="D14:D34">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>LEFT($D14,1)="✔"</formula>
     </cfRule>
@@ -3572,7 +3543,7 @@
       <formula>$D14="LOCKED"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="38">
+  <dataValidations count="36">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Stamp the time" prompt="Press Ctrl+Shift+: to type the current time." sqref="C6"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Stamp the time" prompt="Press Ctrl+Shift+: to type the current time." sqref="C7"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Type your answer" prompt="Type keys joined with +, like Ctrl+Shift+L. For a function, type its name, like SUMIFS. Case and spaces don't matter." sqref="C14"/>
@@ -3603,8 +3574,8 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Need a hint?" prompt="Pick 'Show hint' (Alt+Down). This question then gives 5 XP instead of 10." sqref="E20">
       <formula1>"Show hint"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Type your answer" prompt="Type keys joined with +, like Ctrl+Shift+L. For a function, type its name, like SUMIFS. Case and spaces don't matter." sqref="C21"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Need a hint?" prompt="Pick 'Show hint' (Alt+Down). This question then gives 5 XP instead of 10." sqref="E21">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Type what you found" prompt="Do the move in the arena, then type the word or number you found here." sqref="C25"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Need a hint?" prompt="Pick 'Show hint' (Alt+Down). This question then gives 5 XP instead of 10." sqref="E25">
       <formula1>"Show hint"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Type what you found" prompt="Do the move in the arena, then type the word or number you found here." sqref="C26"/>
@@ -3643,13 +3614,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Need a hint?" prompt="Pick 'Show hint' (Alt+Down). This question then gives 5 XP instead of 10." sqref="E34">
       <formula1>"Show hint"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Type what you found" prompt="Do the move in the arena, then type the word or number you found here." sqref="C35"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Need a hint?" prompt="Pick 'Show hint' (Alt+Down). This question then gives 5 XP instead of 10." sqref="E35">
-      <formula1>"Show hint"</formula1>
-    </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B24" location="'Boss Arena'!A1" display="▶ Open Boss Arena (or press Ctrl+PgDn)"/>
+    <hyperlink ref="B23" location="'Boss Arena'!A1" display="▶ Open Boss Arena (or press Ctrl+PgDn)"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
@@ -17012,7 +16979,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -17020,245 +16987,245 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="6" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="35.5" customHeight="1">
       <c r="A5" s="18" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>24</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="35.5" customHeight="1">
       <c r="A6" s="18" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="35.5" customHeight="1">
       <c r="A7" s="18" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>30</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="35.5" customHeight="1">
       <c r="A8" s="18" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B8" s="19" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="35.5" customHeight="1">
       <c r="A9" s="18" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>52</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="35.5" customHeight="1">
       <c r="A10" s="18" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>114</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="19.75" customHeight="1">
       <c r="A11" s="18" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>46</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="35.5" customHeight="1">
       <c r="A12" s="18" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>45</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="19.75" customHeight="1">
       <c r="A13" s="18" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>119</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="35.5" customHeight="1">
       <c r="A14" s="18" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B14" s="19" t="s">
         <v>63</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="35.5" customHeight="1">
       <c r="A15" s="18" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="35.5" customHeight="1">
       <c r="A16" s="18" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B16" s="19" t="s">
         <v>199</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="35.5" customHeight="1">
       <c r="A17" s="18" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>57</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="35.5" customHeight="1">
       <c r="A18" s="18" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B18" s="19" t="s">
         <v>44</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="35.5" customHeight="1">
       <c r="A19" s="18" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="35.5" customHeight="1">
       <c r="A20" s="18" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B20" s="19" t="s">
         <v>217</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
   </sheetData>
@@ -17270,7 +17237,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N80"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -18373,82 +18340,79 @@
     </row>
     <row r="70" spans="1:9">
       <c r="A70" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B70" t="s">
-        <v>133</v>
-      </c>
-      <c r="E70" t="s">
-        <v>150</v>
-      </c>
-      <c r="F70" t="s">
-        <v>151</v>
+        <v>386</v>
+      </c>
+      <c r="C70" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="71" spans="1:9">
       <c r="A71" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B71" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C71" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="72" spans="1:9">
       <c r="A72" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B72" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C72" t="s">
-        <v>334</v>
+        <v>361</v>
       </c>
     </row>
     <row r="73" spans="1:9">
       <c r="A73" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B73" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C73" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="74" spans="1:9">
       <c r="A74" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B74" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C74" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="75" spans="1:9">
       <c r="A75" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B75" t="s">
-        <v>400</v>
-      </c>
-      <c r="C75" t="s">
-        <v>360</v>
+        <v>401</v>
+      </c>
+      <c r="C75">
+        <v>1707</v>
       </c>
     </row>
     <row r="76" spans="1:9">
       <c r="A76" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B76" t="s">
-        <v>403</v>
+        <v>319</v>
       </c>
       <c r="C76">
-        <v>1707</v>
+        <v>247</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -18456,42 +18420,31 @@
         <v>405</v>
       </c>
       <c r="B77" t="s">
-        <v>319</v>
+        <v>406</v>
       </c>
       <c r="C77">
-        <v>247</v>
+        <v>64</v>
       </c>
     </row>
     <row r="78" spans="1:9">
       <c r="A78" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B78" t="s">
-        <v>408</v>
-      </c>
-      <c r="C78">
-        <v>64</v>
+        <v>409</v>
+      </c>
+      <c r="C78" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="79" spans="1:9">
       <c r="A79" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B79" t="s">
-        <v>411</v>
-      </c>
-      <c r="C79" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9">
-      <c r="A80" t="s">
-        <v>413</v>
-      </c>
-      <c r="B80" t="s">
         <v>322</v>
       </c>
-      <c r="C80">
+      <c r="C79">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: address final review — spill-proof column check, date stamps survive midnight, answerable Training questions
- column_hidden: INDEX(CELL("width"),1)=0; CELL("width") returns two items in Excel 365 and spilled
  into the Hint? picker (picking a hint then broke the world's scoring). Harness now asserts no
  learner-facing formula spills.
- today_constant: accept a whole-day date constant from the build date up to TODAY(), so a Ctrl+;
  stamp keeps its tick the next day.
- Course.pick: when an item's label isn't itself an accepted answer, ask 'Which move is this? <what>'
  so the right option always answers the question; dropdown questions never say 'Type'.
- SelfCheck result is IFERROR-guarded like every other result formula.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EaSHWrLVjcRFSEFZAsuapw
</commit_message>
<xml_diff>
--- a/workbooks/01 Shortcuts 1 - Navigate and Select.xlsx
+++ b/workbooks/01 Shortcuts 1 - Navigate and Select.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="490">
   <si>
     <t>Challenge</t>
   </si>
@@ -749,82 +749,91 @@
     <t>A function key, or Ctrl plus G.</t>
   </si>
   <si>
+    <t>Which move is this? Open Go To: type an address or a name and jump there.</t>
+  </si>
+  <si>
+    <t>S1-2 Teleport T2</t>
+  </si>
+  <si>
+    <t>Ctrl plus Page Down.</t>
+  </si>
+  <si>
+    <t>Which keys move to the next sheet?</t>
+  </si>
+  <si>
+    <t>S1-2 Teleport T3</t>
+  </si>
+  <si>
+    <t>Ctrl plus Page Up.</t>
+  </si>
+  <si>
+    <t>Which keys move to the previous sheet?</t>
+  </si>
+  <si>
+    <t>S1-2 Teleport T4</t>
+  </si>
+  <si>
+    <t>Page Down.</t>
+  </si>
+  <si>
+    <t>Which move is this? Scroll one screen down / up.</t>
+  </si>
+  <si>
+    <t>S1-2 Teleport T5</t>
+  </si>
+  <si>
+    <t>Alt plus Page Down.</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t>Which move is this? Scroll one screen right / left.</t>
+  </si>
+  <si>
+    <t>▶ Open S1-2 Arena (or press Ctrl+PgDn)</t>
+  </si>
+  <si>
+    <t>S1-2 Teleport C1</t>
+  </si>
+  <si>
+    <t>CTRL+G</t>
+  </si>
+  <si>
+    <t>F5</t>
+  </si>
+  <si>
     <t>Which key opens the Go To box?</t>
   </si>
   <si>
-    <t>S1-2 Teleport T2</t>
-  </si>
-  <si>
-    <t>Ctrl plus Page Down.</t>
-  </si>
-  <si>
-    <t>Which keys move to the next sheet?</t>
-  </si>
-  <si>
-    <t>S1-2 Teleport T3</t>
-  </si>
-  <si>
-    <t>Ctrl plus Page Up.</t>
-  </si>
-  <si>
-    <t>Which keys move to the previous sheet?</t>
-  </si>
-  <si>
-    <t>S1-2 Teleport T4</t>
-  </si>
-  <si>
-    <t>Page Down.</t>
+    <t>S1-2 Teleport C2</t>
+  </si>
+  <si>
+    <t>CTRL+PGDN</t>
+  </si>
+  <si>
+    <t>S1-2 Teleport C3</t>
+  </si>
+  <si>
+    <t>CTRL+PGUP</t>
+  </si>
+  <si>
+    <t>S1-2 Teleport C4</t>
+  </si>
+  <si>
+    <t>PGDN</t>
   </si>
   <si>
     <t>Which key scrolls one screen down?</t>
   </si>
   <si>
-    <t>S1-2 Teleport T5</t>
-  </si>
-  <si>
-    <t>Alt plus Page Down.</t>
-  </si>
-  <si>
-    <t>T5</t>
+    <t>S1-2 Teleport C5</t>
+  </si>
+  <si>
+    <t>ALT+PGDN</t>
   </si>
   <si>
     <t>Which keys scroll one screen to the right?</t>
-  </si>
-  <si>
-    <t>▶ Open S1-2 Arena (or press Ctrl+PgDn)</t>
-  </si>
-  <si>
-    <t>S1-2 Teleport C1</t>
-  </si>
-  <si>
-    <t>CTRL+G</t>
-  </si>
-  <si>
-    <t>F5</t>
-  </si>
-  <si>
-    <t>S1-2 Teleport C2</t>
-  </si>
-  <si>
-    <t>CTRL+PGDN</t>
-  </si>
-  <si>
-    <t>S1-2 Teleport C3</t>
-  </si>
-  <si>
-    <t>CTRL+PGUP</t>
-  </si>
-  <si>
-    <t>S1-2 Teleport C4</t>
-  </si>
-  <si>
-    <t>PGDN</t>
-  </si>
-  <si>
-    <t>S1-2 Teleport C5</t>
-  </si>
-  <si>
-    <t>ALT+PGDN</t>
   </si>
   <si>
     <t>S1-2 Teleport C6</t>
@@ -2714,7 +2723,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2724,12 +2733,12 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -2739,32 +2748,32 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="5" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="5" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="5" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="5" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="5" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="4" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -2774,30 +2783,30 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="6" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="7" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="C13" s="9" cm="1" t="str">
         <f t="array" ref="C13">SUM('S1-1 Warp Zones'!$G$17:$G$33)&amp;" / 130"</f>
@@ -2812,15 +2821,15 @@
         <v>NEW</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="7" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="C14" s="9" cm="1" t="str">
         <f t="array" ref="C14">SUM('S1-2 Teleport'!$G$15:$G$39)&amp;" / 180"</f>
@@ -2835,15 +2844,15 @@
         <v>NEW</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="7" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="C15" s="9" cm="1" t="str">
         <f t="array" ref="C15">SUM('S1-3 Lasso'!$G$14:$G$37)&amp;" / 170"</f>
@@ -2858,15 +2867,15 @@
         <v>NEW</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="7" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="C16" s="9" cm="1" t="str">
         <f t="array" ref="C16">SUM('S1-4 Grab'!$G$13:$G$32)&amp;" / 130"</f>
@@ -2881,15 +2890,15 @@
         <v>NEW</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="7" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="C17" s="9" cm="1" t="str">
         <f t="array" ref="C17">SUM(Boss!$G$14:$G$34)&amp;" / 170"</f>
@@ -2904,12 +2913,12 @@
         <v>LOCKED</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="7" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B19" s="12" cm="1" t="str">
         <f t="array" ref="B19">(SUM('S1-1 Warp Zones'!$G$17:$G$33)+SUM('S1-2 Teleport'!$G$15:$G$39)+SUM('S1-3 Lasso'!$G$14:$G$37)+SUM('S1-4 Grab'!$G$13:$G$32)+SUM(Boss!$G$14:$G$34))&amp;" / 780"</f>
@@ -2918,19 +2927,19 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="7" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B20" s="12" cm="1" t="str">
         <f t="array" ref="B20">_xlfn.LET(_xlpm.p,(SUM('S1-1 Warp Zones'!$G$17:$G$33)+SUM('S1-2 Teleport'!$G$15:$G$39)+SUM('S1-3 Lasso'!$G$14:$G$37)+SUM('S1-4 Grab'!$G$13:$G$32)+SUM(Boss!$G$14:$G$34))/780,IF(AND(_xlpm.p&gt;=1,ISNUMBER(Boss!$C$8),Boss!$C$8&lt;=10),"S",IF(_xlpm.p&gt;=0.9,"A",IF(_xlpm.p&gt;=0.75,"B",IF(_xlpm.p&gt;=0.5,"C","D")))))</f>
         <v>D</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="7" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B21" s="12" cm="1" t="str">
         <f t="array" ref="B21">IF(ISNUMBER(Boss!$C$8),Boss!$C$8&amp;" min (par 10)","—")</f>
@@ -2939,7 +2948,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="7" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="B22" s="12" cm="1" t="str">
         <f t="array" ref="B22">IFERROR(INDEX($A$13:$A$16,MATCH("☆☆☆",$D$13:$D$16,0))&amp;" "&amp;INDEX($B$13:$B$16,MATCH("☆☆☆",$D$13:$D$16,0)),IF(Boss!$C$10="OPEN","the Boss","All clear! Aim for rank S"))</f>
@@ -2948,7 +2957,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="13" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
     </row>
   </sheetData>
@@ -2985,7 +2994,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2996,7 +3005,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="26" customHeight="1">
@@ -3015,7 +3024,7 @@
     </row>
     <row r="5" spans="1:7" ht="22" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -3026,19 +3035,19 @@
     </row>
     <row r="6" spans="1:7">
       <c r="B6" s="7" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="C6" s="29"/>
     </row>
     <row r="7" spans="1:7">
       <c r="B7" s="7" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C7" s="29"/>
     </row>
     <row r="8" spans="1:7">
       <c r="B8" s="7" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C8" s="30" cm="1" t="str">
         <f t="array" ref="C8">IF(OR(C6="",C7=""),"",ROUND(MOD(C7-C6,1)*1440,0))</f>
@@ -3047,7 +3056,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="B9" s="7" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C9" s="30">
         <v>10</v>
@@ -3055,7 +3064,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="B10" s="7" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="C10" s="12" cm="1" t="str">
         <f t="array" ref="C10">IF(AND(SUM('S1-1 Warp Zones'!$G$17:$G$33)&gt;=130*0.5,SUM('S1-2 Teleport'!$G$15:$G$39)&gt;=180*0.5,SUM('S1-3 Lasso'!$G$14:$G$37)&gt;=170*0.5,SUM('S1-4 Grab'!$G$13:$G$32)&gt;=130*0.5),"OPEN","LOCKED")</f>
@@ -3068,7 +3077,7 @@
     </row>
     <row r="12" spans="1:7" ht="22" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -3102,7 +3111,7 @@
     </row>
     <row r="14" spans="1:7" ht="35.5" customHeight="1">
       <c r="A14" s="18" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B14" s="31" cm="1" t="str">
         <f t="array" ref="B14">IF($C$10="OPEN","Which keys select the entire row?  (from S1-4 Grab)","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3125,7 +3134,7 @@
     </row>
     <row r="15" spans="1:7" ht="35.5" customHeight="1">
       <c r="A15" s="18" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B15" s="31" cm="1" t="str">
         <f t="array" ref="B15">IF($C$10="OPEN","Which keys select the entire column?  (from S1-4 Grab)","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3148,7 +3157,7 @@
     </row>
     <row r="16" spans="1:7" ht="51.25" customHeight="1">
       <c r="A16" s="18" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B16" s="31" cm="1" t="str">
         <f t="array" ref="B16">IF($C$10="OPEN","Which keys select the current data block (and the whole sheet if you keep pressing)?  (from S1-4 Grab)","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3171,7 +3180,7 @@
     </row>
     <row r="17" spans="1:7" ht="35.5" customHeight="1">
       <c r="A17" s="18" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B17" s="31" cm="1" t="str">
         <f t="array" ref="B17">IF($C$10="OPEN","Which keys jump to the edge of the current data block (any direction)?  (from S1-1 Warp Zones)","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3217,7 +3226,7 @@
     </row>
     <row r="19" spans="1:7" ht="35.5" customHeight="1">
       <c r="A19" s="18" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="B19" s="31" cm="1" t="str">
         <f t="array" ref="B19">IF($C$10="OPEN","Which keys jump to the last used cell on the sheet?  (from S1-1 Warp Zones)","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3240,7 +3249,7 @@
     </row>
     <row r="20" spans="1:7" ht="35.5" customHeight="1">
       <c r="A20" s="18" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B20" s="31" cm="1" t="str">
         <f t="array" ref="B20">IF($C$10="OPEN","Which single key moves to column A of the current row?  (from S1-1 Warp Zones)","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3263,7 +3272,7 @@
     </row>
     <row r="22" spans="1:7" ht="22" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -3274,7 +3283,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="B23" s="11" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -3302,7 +3311,7 @@
     </row>
     <row r="25" spans="1:7" ht="35.5" customHeight="1">
       <c r="A25" s="18" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B25" s="31" cm="1" t="str">
         <f t="array" ref="B25">IF($C$10="OPEN","In the Boss Arena, click B6 and press Ctrl+↓. Type the word at the end of the long trail.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3325,7 +3334,7 @@
     </row>
     <row r="26" spans="1:7" ht="35.5" customHeight="1">
       <c r="A26" s="18" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="B26" s="31" cm="1" t="str">
         <f t="array" ref="B26">IF($C$10="OPEN","Click D6 and keep pressing Ctrl+↓ across the gaps. Type the word you reach.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3348,7 +3357,7 @@
     </row>
     <row r="27" spans="1:7" ht="35.5" customHeight="1">
       <c r="A27" s="18" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B27" s="31" cm="1" t="str">
         <f t="array" ref="B27">IF($C$10="OPEN","Press F5, go to J1200, then press Ctrl+→. Type the word you land on.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3371,7 +3380,7 @@
     </row>
     <row r="28" spans="1:7" ht="35.5" customHeight="1">
       <c r="A28" s="18" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B28" s="31" cm="1" t="str">
         <f t="array" ref="B28">IF($C$10="OPEN","Press Ctrl+End. Type the word in the last used cell.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3394,7 +3403,7 @@
     </row>
     <row r="29" spans="1:7" ht="35.5" customHeight="1">
       <c r="A29" s="18" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B29" s="31" cm="1" t="str">
         <f t="array" ref="B29">IF($C$10="OPEN","Press F5 (or Ctrl+G) and go to Q900. Type the word there.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3417,7 +3426,7 @@
     </row>
     <row r="30" spans="1:7" ht="35.5" customHeight="1">
       <c r="A30" s="18" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B30" s="31" cm="1" t="str">
         <f t="array" ref="B30">IF($C$10="OPEN","Click F6 and press Ctrl+Shift+↓ to select all ENERGY values. Type the status-bar Sum.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3440,7 +3449,7 @@
     </row>
     <row r="31" spans="1:7" ht="35.5" customHeight="1">
       <c r="A31" s="18" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B31" s="31" cm="1" t="str">
         <f t="array" ref="B31">IF($C$10="OPEN","Click any cell in column H and press Ctrl+Space. Type the status-bar Sum.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3463,7 +3472,7 @@
     </row>
     <row r="32" spans="1:7" ht="51.25" customHeight="1">
       <c r="A32" s="18" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B32" s="31" cm="1" t="str">
         <f t="array" ref="B32">IF($C$10="OPEN","Click inside the MOONS table (it starts at L40) and press Ctrl+A once. Type the status-bar Count.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3486,7 +3495,7 @@
     </row>
     <row r="33" spans="1:7" ht="35.5" customHeight="1">
       <c r="A33" s="18" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B33" s="31" cm="1" t="str">
         <f t="array" ref="B33">IF($C$10="OPEN","Click S40 (START) and press Home. Type the word in the cell you land on.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3509,7 +3518,7 @@
     </row>
     <row r="34" spans="1:7" ht="35.5" customHeight="1">
       <c r="A34" s="18" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B34" s="31" cm="1" t="str">
         <f t="array" ref="B34">IF($C$10="OPEN","Click any cell in row 20 and press Shift+Space. Type the status-bar Count.","LOCKED · earn ★ on every stage to open the Boss gate")</f>
@@ -3634,7 +3643,7 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3647,24 +3656,24 @@
         <v>6</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="B5" s="28" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D5" s="28" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="H5" s="28" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3880,13 +3889,13 @@
         <v>5</v>
       </c>
       <c r="L20" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="N20" s="5">
         <v>8</v>
       </c>
       <c r="P20" s="5" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="R20" s="5">
         <v>13</v>
@@ -4120,7 +4129,7 @@
         <v>18</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="39" spans="1:19">
@@ -4136,7 +4145,7 @@
     </row>
     <row r="40" spans="1:19">
       <c r="A40" s="5" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B40" s="5">
         <v>35</v>
@@ -4148,19 +4157,19 @@
         <v>11</v>
       </c>
       <c r="L40" s="28" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="M40" s="28" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="N40" s="28" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="O40" s="28" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="S40" s="7" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="41" spans="1:19">
@@ -4174,16 +4183,16 @@
         <v>22</v>
       </c>
       <c r="L41" s="5" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="N41" s="5">
         <v>3474</v>
       </c>
       <c r="O41" s="5" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="42" spans="1:19">
@@ -4197,10 +4206,10 @@
         <v>4</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="M42" s="5" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="N42" s="5">
         <v>22</v>
@@ -4220,10 +4229,10 @@
         <v>15</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="M43" s="5" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="N43" s="5">
         <v>12</v>
@@ -4243,10 +4252,10 @@
         <v>26</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="M44" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="N44" s="5">
         <v>3643</v>
@@ -4266,10 +4275,10 @@
         <v>8</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="M45" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="N45" s="5">
         <v>3122</v>
@@ -4289,10 +4298,10 @@
         <v>19</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="M46" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="N46" s="5">
         <v>5268</v>
@@ -4312,10 +4321,10 @@
         <v>30</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="M47" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="N47" s="5">
         <v>4821</v>
@@ -4335,10 +4344,10 @@
         <v>12</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="M48" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="N48" s="5">
         <v>5150</v>
@@ -4358,10 +4367,10 @@
         <v>23</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="M49" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="N49" s="5">
         <v>1527</v>
@@ -4381,10 +4390,10 @@
         <v>5</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="M50" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="N50" s="5">
         <v>1469</v>
@@ -4401,10 +4410,10 @@
         <v>16</v>
       </c>
       <c r="L51" s="5" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="M51" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="N51" s="5">
         <v>1123</v>
@@ -4421,10 +4430,10 @@
         <v>27</v>
       </c>
       <c r="L52" s="5" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="M52" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="N52" s="5">
         <v>472</v>
@@ -4441,10 +4450,10 @@
         <v>9</v>
       </c>
       <c r="L53" s="5" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="M53" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="N53" s="5">
         <v>1158</v>
@@ -4461,10 +4470,10 @@
         <v>20</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="N54" s="5">
         <v>2707</v>
@@ -4481,10 +4490,10 @@
         <v>31</v>
       </c>
       <c r="L55" s="5" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="M55" s="5" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="N55" s="5">
         <v>1212</v>
@@ -5901,7 +5910,7 @@
         <v>295</v>
       </c>
       <c r="D300" s="5" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="301" spans="2:4">
@@ -8904,7 +8913,7 @@
         <v>895</v>
       </c>
       <c r="Q900" s="5" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="901" spans="2:17">
@@ -10443,7 +10452,7 @@
         <v>11</v>
       </c>
       <c r="U1200" s="5" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="1201" spans="2:2">
@@ -16948,10 +16957,10 @@
     </row>
     <row r="2501" spans="2:21">
       <c r="B2501" s="5" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="U2501" s="5" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -16979,7 +16988,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -16987,245 +16996,245 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="6" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="35.5" customHeight="1">
       <c r="A5" s="18" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>24</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="35.5" customHeight="1">
       <c r="A6" s="18" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="35.5" customHeight="1">
       <c r="A7" s="18" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>30</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="35.5" customHeight="1">
       <c r="A8" s="18" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B8" s="19" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="35.5" customHeight="1">
       <c r="A9" s="18" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>52</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="35.5" customHeight="1">
       <c r="A10" s="18" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>114</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="19.75" customHeight="1">
       <c r="A11" s="18" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>46</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="35.5" customHeight="1">
       <c r="A12" s="18" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>45</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="19.75" customHeight="1">
       <c r="A13" s="18" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>119</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="35.5" customHeight="1">
       <c r="A14" s="18" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B14" s="19" t="s">
         <v>63</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="35.5" customHeight="1">
       <c r="A15" s="18" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="35.5" customHeight="1">
       <c r="A16" s="18" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="35.5" customHeight="1">
       <c r="A17" s="18" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>57</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="35.5" customHeight="1">
       <c r="A18" s="18" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B18" s="19" t="s">
         <v>44</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="35.5" customHeight="1">
       <c r="A19" s="18" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="35.5" customHeight="1">
       <c r="A20" s="18" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
   </sheetData>
@@ -17644,54 +17653,54 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B25" t="s">
         <v>136</v>
       </c>
       <c r="E25" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B26" t="s">
         <v>139</v>
       </c>
       <c r="E26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B27" t="s">
         <v>142</v>
       </c>
       <c r="E27" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B28" t="s">
         <v>145</v>
       </c>
       <c r="E28" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B29" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C29" t="s">
         <v>110</v>
@@ -17699,10 +17708,10 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B30" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C30" t="s">
         <v>111</v>
@@ -17710,10 +17719,10 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B31" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C31" t="s">
         <v>107</v>
@@ -17721,10 +17730,10 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B32" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C32" t="s">
         <v>7</v>
@@ -17732,7 +17741,7 @@
     </row>
     <row r="33" spans="1:14">
       <c r="A33" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B33" t="s">
         <v>133</v>
@@ -17746,54 +17755,54 @@
     </row>
     <row r="34" spans="1:14">
       <c r="A34" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B34" t="s">
         <v>136</v>
       </c>
       <c r="E34" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:14">
       <c r="A35" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B35" t="s">
         <v>139</v>
       </c>
       <c r="E35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="36" spans="1:14">
       <c r="A36" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B36" t="s">
         <v>142</v>
       </c>
       <c r="E36" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="37" spans="1:14">
       <c r="A37" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B37" t="s">
         <v>145</v>
       </c>
       <c r="E37" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="38" spans="1:14">
       <c r="A38" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B38" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C38" t="s">
         <v>63</v>
@@ -17813,10 +17822,10 @@
     </row>
     <row r="39" spans="1:14">
       <c r="A39" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B39" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C39" t="s">
         <v>58</v>
@@ -17825,7 +17834,7 @@
         <v>58</v>
       </c>
       <c r="F39" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G39" t="s">
         <v>63</v>
@@ -17836,16 +17845,16 @@
     </row>
     <row r="40" spans="1:14">
       <c r="A40" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B40" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C40" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E40" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F40" t="s">
         <v>51</v>
@@ -17859,10 +17868,10 @@
     </row>
     <row r="41" spans="1:14">
       <c r="A41" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B41" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C41" t="s">
         <v>57</v>
@@ -17882,99 +17891,99 @@
     </row>
     <row r="42" spans="1:14">
       <c r="A42" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B42" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="E42" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F42" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="G42" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="H42" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="I42" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="43" spans="1:14">
       <c r="A43" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B43" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E43" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F43" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="G43" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="H43" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="I43" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="J43" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="K43" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="L43" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="M43" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="N43" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="44" spans="1:14">
       <c r="A44" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B44" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E44" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F44" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="45" spans="1:14">
       <c r="A45" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B45" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E45" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F45" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="46" spans="1:14">
       <c r="A46" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B46" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C46">
         <v>2417</v>
@@ -17982,10 +17991,10 @@
     </row>
     <row r="47" spans="1:14">
       <c r="A47" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B47" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C47">
         <v>64</v>
@@ -17993,10 +18002,10 @@
     </row>
     <row r="48" spans="1:14">
       <c r="A48" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B48" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C48">
         <v>34</v>
@@ -18004,10 +18013,10 @@
     </row>
     <row r="49" spans="1:14">
       <c r="A49" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B49" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C49">
         <v>42</v>
@@ -18015,105 +18024,105 @@
     </row>
     <row r="50" spans="1:14">
       <c r="A50" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B50" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="E50" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F50" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="G50" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="H50" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="I50" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="51" spans="1:14">
       <c r="A51" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B51" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E51" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F51" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="G51" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="H51" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="I51" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="J51" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="K51" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="L51" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="M51" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="N51" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="52" spans="1:14">
       <c r="A52" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B52" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E52" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F52" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="53" spans="1:14">
       <c r="A53" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B53" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E53" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F53" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="54" spans="1:14">
       <c r="A54" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B54" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="C54" t="s">
         <v>44</v>
       </c>
       <c r="E54" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F54" t="s">
         <v>46</v>
@@ -18127,10 +18136,10 @@
     </row>
     <row r="55" spans="1:14">
       <c r="A55" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B55" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C55" t="s">
         <v>51</v>
@@ -18139,7 +18148,7 @@
         <v>51</v>
       </c>
       <c r="F55" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G55" t="s">
         <v>46</v>
@@ -18150,13 +18159,13 @@
     </row>
     <row r="56" spans="1:14">
       <c r="A56" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B56" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C56" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="E56" t="s">
         <v>46</v>
@@ -18165,7 +18174,7 @@
         <v>45</v>
       </c>
       <c r="G56" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="H56" t="s">
         <v>44</v>
@@ -18173,49 +18182,49 @@
     </row>
     <row r="57" spans="1:14">
       <c r="A57" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B57" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E57" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="58" spans="1:14">
       <c r="A58" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B58" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="E58" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="59" spans="1:14">
       <c r="A59" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B59" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E59" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F59" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="G59" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="60" spans="1:14">
       <c r="A60" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B60" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C60">
         <v>462</v>
@@ -18223,10 +18232,10 @@
     </row>
     <row r="61" spans="1:14">
       <c r="A61" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B61" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C61">
         <v>6</v>
@@ -18234,10 +18243,10 @@
     </row>
     <row r="62" spans="1:14">
       <c r="A62" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B62" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C62">
         <v>52</v>
@@ -18245,46 +18254,46 @@
     </row>
     <row r="63" spans="1:14">
       <c r="A63" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B63" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E63" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="64" spans="1:14">
       <c r="A64" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B64" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="E64" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="65" spans="1:9">
       <c r="A65" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B65" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E65" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F65" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="G65" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="66" spans="1:9">
       <c r="A66" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B66" t="s">
         <v>43</v>
@@ -18307,7 +18316,7 @@
     </row>
     <row r="67" spans="1:9">
       <c r="A67" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B67" t="s">
         <v>50</v>
@@ -18318,7 +18327,7 @@
     </row>
     <row r="68" spans="1:9">
       <c r="A68" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B68" t="s">
         <v>56</v>
@@ -18329,7 +18338,7 @@
     </row>
     <row r="69" spans="1:9">
       <c r="A69" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B69" t="s">
         <v>62</v>
@@ -18340,65 +18349,65 @@
     </row>
     <row r="70" spans="1:9">
       <c r="A70" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B70" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C70" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="71" spans="1:9">
       <c r="A71" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B71" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C71" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="72" spans="1:9">
       <c r="A72" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B72" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="C72" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="73" spans="1:9">
       <c r="A73" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B73" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="C73" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="74" spans="1:9">
       <c r="A74" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B74" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="C74" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="75" spans="1:9">
       <c r="A75" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B75" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="C75">
         <v>1707</v>
@@ -18406,10 +18415,10 @@
     </row>
     <row r="76" spans="1:9">
       <c r="A76" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B76" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C76">
         <v>247</v>
@@ -18417,10 +18426,10 @@
     </row>
     <row r="77" spans="1:9">
       <c r="A77" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B77" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="C77">
         <v>64</v>
@@ -18428,21 +18437,21 @@
     </row>
     <row r="78" spans="1:9">
       <c r="A78" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="B78" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="C78" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="79" spans="1:9">
       <c r="A79" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B79" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C79">
         <v>9</v>
@@ -28378,7 +28387,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -28389,7 +28398,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="26" customHeight="1">
@@ -28647,7 +28656,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="19.75" customHeight="1">
+    <row r="22" spans="1:7" ht="35.5" customHeight="1">
       <c r="A22" s="18" t="s">
         <v>47</v>
       </c>
@@ -28713,7 +28722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="19.75" customHeight="1">
+    <row r="25" spans="1:7" ht="35.5" customHeight="1">
       <c r="A25" s="18" t="s">
         <v>64</v>
       </c>
@@ -28735,7 +28744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="19.75" customHeight="1">
+    <row r="26" spans="1:7" ht="35.5" customHeight="1">
       <c r="A26" s="18" t="s">
         <v>146</v>
       </c>
@@ -28801,7 +28810,7 @@
         <v>74</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
       <c r="C31" s="21"/>
       <c r="D31" s="22" cm="1" t="str">
@@ -28867,7 +28876,7 @@
         <v>83</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="C34" s="21"/>
       <c r="D34" s="22" cm="1" t="str">
@@ -28889,7 +28898,7 @@
         <v>86</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="C35" s="21"/>
       <c r="D35" s="22" cm="1" t="str">
@@ -28911,7 +28920,7 @@
         <v>90</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C36" s="21"/>
       <c r="D36" s="22" cm="1" t="str">
@@ -28933,7 +28942,7 @@
         <v>94</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37" s="22" cm="1" t="str">
@@ -28955,7 +28964,7 @@
         <v>98</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C38" s="21"/>
       <c r="D38" s="22" cm="1" t="str">
@@ -28977,7 +28986,7 @@
         <v>102</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C39" s="21"/>
       <c r="D39" s="22" cm="1" t="str">
@@ -29172,7 +29181,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -29183,7 +29192,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="26" customHeight="1">
@@ -29235,7 +29244,7 @@
         <v>22</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>63</v>
@@ -29246,7 +29255,7 @@
         <v>25</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>58</v>
@@ -29257,10 +29266,10 @@
         <v>28</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="51.25" customHeight="1">
@@ -29268,7 +29277,7 @@
         <v>31</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>57</v>
@@ -29313,7 +29322,7 @@
         <v>121</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C14" s="21"/>
       <c r="D14" s="22" cm="1" t="str">
@@ -29335,7 +29344,7 @@
         <v>124</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C15" s="21"/>
       <c r="D15" s="22" cm="1" t="str">
@@ -29357,7 +29366,7 @@
         <v>127</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C16" s="21"/>
       <c r="D16" s="22" cm="1" t="str">
@@ -29379,7 +29388,7 @@
         <v>130</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C17" s="21"/>
       <c r="D17" s="22" cm="1" t="str">
@@ -29398,10 +29407,10 @@
     </row>
     <row r="18" spans="1:7" ht="35.5" customHeight="1">
       <c r="A18" s="18" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C18" s="21"/>
       <c r="D18" s="22" cm="1" t="str">
@@ -29457,7 +29466,7 @@
         <v>47</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C22" s="21"/>
       <c r="D22" s="22" cm="1" t="str">
@@ -29479,7 +29488,7 @@
         <v>53</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C23" s="21"/>
       <c r="D23" s="22" cm="1" t="str">
@@ -29501,7 +29510,7 @@
         <v>59</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C24" s="21"/>
       <c r="D24" s="22" cm="1" t="str">
@@ -29523,7 +29532,7 @@
         <v>64</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C25" s="21"/>
       <c r="D25" s="22" cm="1" t="str">
@@ -29553,7 +29562,7 @@
     </row>
     <row r="28" spans="1:7">
       <c r="B28" s="11" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -29584,7 +29593,7 @@
         <v>74</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C30" s="21"/>
       <c r="D30" s="22" cm="1" t="str">
@@ -29606,7 +29615,7 @@
         <v>77</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C31" s="21"/>
       <c r="D31" s="22" cm="1" t="str">
@@ -29628,7 +29637,7 @@
         <v>80</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C32" s="21"/>
       <c r="D32" s="22" cm="1" t="str">
@@ -29650,7 +29659,7 @@
         <v>83</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C33" s="21"/>
       <c r="D33" s="22" cm="1" t="str">
@@ -29672,7 +29681,7 @@
         <v>86</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C34" s="21"/>
       <c r="D34" s="22" cm="1" t="str">
@@ -29694,7 +29703,7 @@
         <v>90</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C35" s="21"/>
       <c r="D35" s="22" cm="1" t="str">
@@ -29716,7 +29725,7 @@
         <v>94</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C36" s="21"/>
       <c r="D36" s="22" cm="1" t="str">
@@ -29738,7 +29747,7 @@
         <v>98</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37" s="22" cm="1" t="str">
@@ -29865,7 +29874,7 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -29878,27 +29887,27 @@
         <v>6</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="B5" s="28" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="H5" s="28" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -29906,7 +29915,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="E6" s="5">
         <v>4</v>
@@ -29915,7 +29924,7 @@
         <v>120</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -29923,7 +29932,7 @@
         <v>15</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E7" s="5">
         <v>6</v>
@@ -29932,7 +29941,7 @@
         <v>95</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -29940,7 +29949,7 @@
         <v>22</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E8" s="5">
         <v>3</v>
@@ -29949,7 +29958,7 @@
         <v>140</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -29957,7 +29966,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E9" s="5">
         <v>8</v>
@@ -29966,7 +29975,7 @@
         <v>210</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -29974,7 +29983,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E10" s="5">
         <v>2</v>
@@ -29988,7 +29997,7 @@
         <v>20</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E11" s="5">
         <v>5</v>
@@ -30002,7 +30011,7 @@
         <v>4</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E12" s="5">
         <v>7</v>
@@ -30016,7 +30025,7 @@
         <v>11</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E13" s="5">
         <v>4</v>
@@ -30030,7 +30039,7 @@
         <v>18</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E14" s="5">
         <v>1</v>
@@ -30044,7 +30053,7 @@
         <v>2</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E15" s="5">
         <v>6</v>
@@ -31031,7 +31040,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -31042,7 +31051,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="26" customHeight="1">
@@ -31094,7 +31103,7 @@
         <v>22</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>44</v>
@@ -31105,7 +31114,7 @@
         <v>25</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>51</v>
@@ -31116,10 +31125,10 @@
         <v>28</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="22" customHeight="1">
@@ -31161,7 +31170,7 @@
         <v>121</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C13" s="21"/>
       <c r="D13" s="22" cm="1" t="str">
@@ -31183,7 +31192,7 @@
         <v>124</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C14" s="21"/>
       <c r="D14" s="22" cm="1" t="str">
@@ -31205,7 +31214,7 @@
         <v>127</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C15" s="21"/>
       <c r="D15" s="22" cm="1" t="str">
@@ -31227,7 +31236,7 @@
         <v>130</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C16" s="21"/>
       <c r="D16" s="22" cm="1" t="str">
@@ -31283,7 +31292,7 @@
         <v>47</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C20" s="21"/>
       <c r="D20" s="22" cm="1" t="str">
@@ -31305,7 +31314,7 @@
         <v>53</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C21" s="21"/>
       <c r="D21" s="22" cm="1" t="str">
@@ -31327,7 +31336,7 @@
         <v>59</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C22" s="21"/>
       <c r="D22" s="22" cm="1" t="str">
@@ -31357,7 +31366,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="B25" s="11" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -31388,7 +31397,7 @@
         <v>74</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C27" s="21"/>
       <c r="D27" s="22" cm="1" t="str">
@@ -31410,7 +31419,7 @@
         <v>77</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C28" s="21"/>
       <c r="D28" s="22" cm="1" t="str">
@@ -31432,7 +31441,7 @@
         <v>80</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C29" s="21"/>
       <c r="D29" s="22" cm="1" t="str">
@@ -31454,7 +31463,7 @@
         <v>83</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C30" s="21"/>
       <c r="D30" s="22" cm="1" t="str">
@@ -31476,7 +31485,7 @@
         <v>86</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C31" s="21"/>
       <c r="D31" s="22" cm="1" t="str">
@@ -31498,7 +31507,7 @@
         <v>90</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C32" s="21"/>
       <c r="D32" s="22" cm="1" t="str">
@@ -31607,7 +31616,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -31620,15 +31629,15 @@
         <v>6</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="F5" s="28" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -31733,7 +31742,7 @@
     </row>
     <row r="30" spans="2:11">
       <c r="B30" s="7" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C30" s="5">
         <v>7</v>
@@ -31742,43 +31751,43 @@
         <v>9</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="I30" s="5">
         <v>4</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="38" spans="2:5">
       <c r="B38" s="7" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="40" spans="2:5">
       <c r="B40" s="28" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C40" s="28" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="D40" s="28" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E40" s="28" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="2:5">
       <c r="B41" s="5" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C41" s="5">
         <v>0</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E41" s="5">
         <v>4223</v>
@@ -31786,13 +31795,13 @@
     </row>
     <row r="42" spans="2:5">
       <c r="B42" s="5" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C42" s="5">
         <v>0</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E42" s="5">
         <v>2802</v>
@@ -31800,13 +31809,13 @@
     </row>
     <row r="43" spans="2:5">
       <c r="B43" s="5" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C43" s="5">
         <v>1</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E43" s="5">
         <v>24</v>
@@ -31814,13 +31823,13 @@
     </row>
     <row r="44" spans="2:5">
       <c r="B44" s="5" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C44" s="5">
         <v>2</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E44" s="5">
         <v>25</v>
@@ -31828,13 +31837,13 @@
     </row>
     <row r="45" spans="2:5">
       <c r="B45" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C45" s="5">
         <v>95</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E45" s="5">
         <v>10</v>
@@ -31842,13 +31851,13 @@
     </row>
     <row r="46" spans="2:5">
       <c r="B46" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C46" s="5">
         <v>146</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E46" s="5">
         <v>11</v>
@@ -31856,13 +31865,13 @@
     </row>
     <row r="47" spans="2:5">
       <c r="B47" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C47" s="5">
         <v>28</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E47" s="5">
         <v>17</v>
@@ -31870,13 +31879,13 @@
     </row>
     <row r="48" spans="2:5">
       <c r="B48" s="5" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C48" s="5">
         <v>16</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E48" s="5">
         <v>16</v>
@@ -31884,13 +31893,13 @@
     </row>
     <row r="49" spans="2:5">
       <c r="B49" s="5" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="C49" s="5">
         <v>0</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E49" s="5">
         <v>9</v>
@@ -31898,13 +31907,13 @@
     </row>
     <row r="50" spans="2:5">
       <c r="B50" s="5" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C50" s="5">
         <v>5</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E50" s="5">
         <v>153</v>
@@ -31912,13 +31921,13 @@
     </row>
     <row r="51" spans="2:5">
       <c r="B51" s="5" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C51" s="5">
         <v>2</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E51" s="5">
         <v>4</v>
@@ -31926,13 +31935,13 @@
     </row>
     <row r="52" spans="2:5">
       <c r="B52" s="5" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C52" s="5">
         <v>1</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E52" s="5">
         <v>26</v>

</xml_diff>

<commit_message>
build: rebuild all 13 workbooks with the minor fixes; spec notes the new behaviors
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EaSHWrLVjcRFSEFZAsuapw
</commit_message>
<xml_diff>
--- a/workbooks/01 Shortcuts 1 - Navigate and Select.xlsx
+++ b/workbooks/01 Shortcuts 1 - Navigate and Select.xlsx
@@ -1930,7 +1930,7 @@
     <t>NEXT UP</t>
   </si>
   <si>
-    <t>Replay a stage: select its yellow answer cells and press Delete. Undo an arena drill with Ctrl+Z.</t>
+    <t>Replay a stage: select a run of its yellow cells (Ctrl+click to add more), then press Delete. Undo an arena drill with Ctrl+Z.</t>
   </si>
   <si>
     <t>CHEAT CODES ▸ NAVIGATE &amp; SELECT</t>
@@ -2951,7 +2951,7 @@
         <v>452</v>
       </c>
       <c r="B22" s="12" cm="1" t="str">
-        <f t="array" ref="B22">IFERROR(INDEX($A$13:$A$16,MATCH("☆☆☆",$D$13:$D$16,0))&amp;" "&amp;INDEX($B$13:$B$16,MATCH("☆☆☆",$D$13:$D$16,0)),IF(Boss!$C$10="OPEN","the Boss","All clear! Aim for rank S"))</f>
+        <f t="array" ref="B22">IFERROR(INDEX($A$13:$A$16,MATCH("☆☆☆",$D$13:$D$16,0))&amp;" "&amp;INDEX($B$13:$B$16,MATCH("☆☆☆",$D$13:$D$16,0)),IF(Start!$E$17="DEFEATED","All clear! Aim for rank S","the Boss"))</f>
         <v>S1-1 Warp Zones</v>
       </c>
     </row>

</xml_diff>